<commit_message>
full site ready all pages built, all function and charts and css and js ready - insert sql and php
</commit_message>
<xml_diff>
--- a/pages to build_ contents each page.xlsx
+++ b/pages to build_ contents each page.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oldwestburyedu-my.sharepoint.com/personal/dshami_oldwestbury_edu/Documents/ONEDRIVE/COLLEGE/OW - SPRING 2026/CS5910 - System Design &amp; Implementation/Project/MILESTONE 3 - website_code_FE-BE-DB/CODE/me/4.19.26/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dani\Documents\repos\CS5910_sys_NYSParks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="8_{463CEA9A-00C6-4923-B0AB-78FB21848E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEBF1A59-22B8-44E4-AA5E-0C2A525F503C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D99931EA-7547-4FBD-9955-872DB901FC0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E7FCEDC8-EB3A-4123-948A-91485DCE2178}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{E7FCEDC8-EB3A-4123-948A-91485DCE2178}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="97">
   <si>
     <t>landing page/ main</t>
   </si>
@@ -202,13 +203,172 @@
   </si>
   <si>
     <t>admin xml</t>
+  </si>
+  <si>
+    <t>final version</t>
+  </si>
+  <si>
+    <t>admin-bookings</t>
+  </si>
+  <si>
+    <t>total 20 pages</t>
+  </si>
+  <si>
+    <t>forgot password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">signup </t>
+  </si>
+  <si>
+    <t>schedule</t>
+  </si>
+  <si>
+    <t>pto req</t>
+  </si>
+  <si>
+    <t>semi-final version</t>
+  </si>
+  <si>
+    <t>semi semi final version</t>
+  </si>
+  <si>
+    <t>logout pt to index</t>
+  </si>
+  <si>
+    <t>Files in staticv4:</t>
+  </si>
+  <si>
+    <t>index.html</t>
+  </si>
+  <si>
+    <t>parks.html</t>
+  </si>
+  <si>
+    <t>events.html</t>
+  </si>
+  <si>
+    <t>map.html</t>
+  </si>
+  <si>
+    <t>ai.html</t>
+  </si>
+  <si>
+    <t>news.html</t>
+  </si>
+  <si>
+    <t>about.html</t>
+  </si>
+  <si>
+    <t>faq.html</t>
+  </si>
+  <si>
+    <t>donate.html</t>
+  </si>
+  <si>
+    <t>login.html</t>
+  </si>
+  <si>
+    <t>forgot-password.html</t>
+  </si>
+  <si>
+    <t>register.html</t>
+  </si>
+  <si>
+    <t>logout.html</t>
+  </si>
+  <si>
+    <t>account.html</t>
+  </si>
+  <si>
+    <t>client-dashboard.html</t>
+  </si>
+  <si>
+    <t>client-create-event.html</t>
+  </si>
+  <si>
+    <t>admin-dashboard.html</t>
+  </si>
+  <si>
+    <t>admin-schedule.html</t>
+  </si>
+  <si>
+    <t>admin-employee-schedule.html</t>
+  </si>
+  <si>
+    <t>admin-pto.html</t>
+  </si>
+  <si>
+    <t>admin-bookings.html</t>
+  </si>
+  <si>
+    <t>admin-xml.html</t>
+  </si>
+  <si>
+    <t>employee-dashboard.html</t>
+  </si>
+  <si>
+    <t>employee-schedule.html</t>
+  </si>
+  <si>
+    <t>employee-pto.html</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">plus shared </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>styles.css</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>app.js</t>
+    </r>
+  </si>
+  <si>
+    <t>Client:</t>
+  </si>
+  <si>
+    <t>Admin:</t>
+  </si>
+  <si>
+    <t>Employee:</t>
+  </si>
+  <si>
+    <t>final final version</t>
+  </si>
+  <si>
+    <t>Main:</t>
+  </si>
+  <si>
+    <t>total pages</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,13 +416,55 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -277,14 +479,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,13 +833,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B453DD6B-30FA-47D6-A01E-C3B26834FBAE}">
-  <dimension ref="A1:AE28"/>
+  <dimension ref="A1:BA41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="43" max="43" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -661,7 +876,7 @@
       </c>
       <c r="V1" s="5"/>
       <c r="W1" s="5"/>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="7" t="s">
         <v>33</v>
       </c>
       <c r="Y1" s="5"/>
@@ -671,12 +886,28 @@
       </c>
       <c r="AB1" s="5"/>
       <c r="AC1" s="5"/>
-      <c r="AD1" s="5" t="s">
+      <c r="AD1" s="9" t="s">
         <v>52</v>
       </c>
       <c r="AE1" s="5"/>
-    </row>
-    <row r="2" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH1" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AM1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ1" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA1" s="14"/>
+    </row>
+    <row r="2" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -701,8 +932,11 @@
       <c r="O2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="X2" s="8"/>
+      <c r="AD2" s="10"/>
+      <c r="AT2" s="12"/>
+    </row>
+    <row r="3" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -730,8 +964,16 @@
       <c r="O3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="X3" s="8"/>
+      <c r="AD3" s="10"/>
+      <c r="AZ3" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="BA3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -750,17 +992,32 @@
       <c r="U4" t="s">
         <v>24</v>
       </c>
-      <c r="X4" t="s">
-        <v>35</v>
+      <c r="X4" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="AA4" t="s">
         <v>27</v>
       </c>
-      <c r="AD4" s="5" t="s">
+      <c r="AD4" s="9" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="AI4" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>27</v>
+      </c>
+      <c r="AQ4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT4" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -779,17 +1036,32 @@
       <c r="U5" t="s">
         <v>6</v>
       </c>
-      <c r="X5" t="s">
-        <v>6</v>
+      <c r="X5" s="8" t="s">
+        <v>3</v>
       </c>
       <c r="AA5" t="s">
         <v>3</v>
       </c>
-      <c r="AD5" s="5" t="s">
+      <c r="AD5" s="9" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>3</v>
+      </c>
+      <c r="AQ5" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="AT5" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="AZ5" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -817,17 +1089,32 @@
       <c r="U6" t="s">
         <v>42</v>
       </c>
-      <c r="X6" t="s">
-        <v>42</v>
+      <c r="X6" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="AA6" t="s">
         <v>4</v>
       </c>
-      <c r="AD6" s="5" t="s">
+      <c r="AD6" s="9" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AQ6" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT6" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ6" s="13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -858,17 +1145,29 @@
       <c r="U7" t="s">
         <v>30</v>
       </c>
-      <c r="X7" t="s">
-        <v>40</v>
+      <c r="X7" s="8" t="s">
+        <v>41</v>
       </c>
       <c r="AA7" t="s">
         <v>41</v>
       </c>
-      <c r="AD7" s="5" t="s">
+      <c r="AI7" s="9" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="8" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AM7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ7" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="AT7" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="AZ7" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -887,17 +1186,32 @@
       <c r="U8" t="s">
         <v>26</v>
       </c>
-      <c r="X8" t="s">
-        <v>39</v>
+      <c r="X8" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="AA8" t="s">
         <v>6</v>
       </c>
-      <c r="AD8" s="5" t="s">
+      <c r="AD8" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AI8" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>6</v>
+      </c>
+      <c r="AQ8" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="AT8" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="AZ8" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -916,17 +1230,30 @@
       <c r="U9" t="s">
         <v>18</v>
       </c>
-      <c r="X9" t="s">
-        <v>36</v>
-      </c>
+      <c r="X9" s="8"/>
       <c r="AA9" t="s">
         <v>17</v>
       </c>
-      <c r="AD9" s="5" t="s">
+      <c r="AD9" s="11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AI9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ9" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="AT9" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="AZ9" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -954,17 +1281,32 @@
       <c r="U10" t="s">
         <v>4</v>
       </c>
-      <c r="X10" t="s">
-        <v>4</v>
+      <c r="X10" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="AA10" t="s">
         <v>35</v>
       </c>
-      <c r="AD10" s="5" t="s">
+      <c r="AD10" s="9" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="11" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>24</v>
+      </c>
+      <c r="AQ10" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="AT10" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="AZ10" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -983,17 +1325,32 @@
       <c r="U11" t="s">
         <v>7</v>
       </c>
-      <c r="X11" t="s">
+      <c r="X11" s="8" t="s">
         <v>7</v>
       </c>
       <c r="AA11" t="s">
         <v>7</v>
       </c>
-      <c r="AD11" s="5" t="s">
+      <c r="AD11" s="9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AI11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>7</v>
+      </c>
+      <c r="AQ11" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="AT11" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="AZ11" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
@@ -1018,17 +1375,30 @@
       <c r="U12" t="s">
         <v>27</v>
       </c>
-      <c r="X12" t="s">
-        <v>27</v>
-      </c>
+      <c r="X12" s="8"/>
       <c r="AA12" t="s">
         <v>18</v>
       </c>
-      <c r="AD12" s="5" t="s">
+      <c r="AD12" s="11" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AI12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>18</v>
+      </c>
+      <c r="AQ12" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="AT12" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="AZ12" s="13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1050,17 +1420,35 @@
       <c r="U13" t="s">
         <v>28</v>
       </c>
-      <c r="X13" t="s">
+      <c r="X13" s="8" t="s">
         <v>28</v>
       </c>
       <c r="AA13" t="s">
         <v>28</v>
       </c>
-      <c r="AD13" s="5" t="s">
+      <c r="AD13" s="9" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI13" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>28</v>
+      </c>
+      <c r="AQ13" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="AT13" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="AZ13" s="13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
@@ -1085,14 +1473,38 @@
       <c r="U14" t="s">
         <v>17</v>
       </c>
+      <c r="X14" s="8" t="s">
+        <v>29</v>
+      </c>
       <c r="AA14" t="s">
         <v>51</v>
       </c>
-      <c r="AD14" s="5" t="s">
+      <c r="AD14" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:31" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AH14" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="AI14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>57</v>
+      </c>
+      <c r="AQ14" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="AR14" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT14" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="AZ14" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:53" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
@@ -1117,113 +1529,402 @@
       <c r="U15" t="s">
         <v>3</v>
       </c>
-      <c r="X15" t="s">
-        <v>3</v>
-      </c>
+      <c r="X15" s="8"/>
       <c r="AA15" t="s">
         <v>50</v>
       </c>
-      <c r="AD15" s="5" t="s">
+      <c r="AD15" s="11" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AI15" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>58</v>
+      </c>
+      <c r="AQ15" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="AT15" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ15" s="13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:53" x14ac:dyDescent="0.25">
       <c r="U16" t="s">
         <v>29</v>
       </c>
-      <c r="X16" t="s">
-        <v>29</v>
-      </c>
+      <c r="X16" s="8"/>
       <c r="AA16" t="s">
         <v>43</v>
       </c>
-      <c r="AD16" s="5" t="s">
+      <c r="AD16" s="11" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="17" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AI16" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ16" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="AT16" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ16" s="13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="21:53" x14ac:dyDescent="0.25">
       <c r="U17" t="s">
         <v>31</v>
       </c>
-      <c r="X17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="21:30" x14ac:dyDescent="0.25">
-      <c r="X18" t="s">
-        <v>37</v>
+      <c r="X17" s="8"/>
+      <c r="AD17" s="10"/>
+      <c r="AM17" t="s">
+        <v>43</v>
+      </c>
+      <c r="AQ17" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT17" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ17" s="13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X18" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="AA18" t="s">
         <v>47</v>
       </c>
-      <c r="AD18" s="5" t="s">
+      <c r="AD18" s="9" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="19" spans="21:30" x14ac:dyDescent="0.25">
-      <c r="X19" t="s">
-        <v>38</v>
+      <c r="AH18" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AI18" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AT18" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="AZ18" s="13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X19" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="AA19" t="s">
         <v>42</v>
       </c>
-      <c r="AD19" s="5" t="s">
+      <c r="AD19" s="9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="21" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AH19" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI19" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="AM19" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ19" t="s">
+        <v>91</v>
+      </c>
+      <c r="AT19" s="13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X20" s="8"/>
+      <c r="AD20" s="10"/>
+      <c r="AH20" s="8"/>
+      <c r="AI20" s="10"/>
+      <c r="AM20" t="s">
+        <v>45</v>
+      </c>
+      <c r="AQ20" s="12"/>
+      <c r="AT20" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="AZ20" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="BA20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X21" s="8" t="s">
+        <v>36</v>
+      </c>
       <c r="AA21" t="s">
         <v>45</v>
       </c>
-      <c r="AD21" s="5" t="s">
+      <c r="AD21" s="9" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="22" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AH21" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="AI21" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>46</v>
+      </c>
+      <c r="AQ21" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT21" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="AZ21" s="12"/>
+    </row>
+    <row r="22" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X22" s="8" t="s">
+        <v>37</v>
+      </c>
       <c r="AA22" t="s">
         <v>46</v>
       </c>
-      <c r="AD22" s="5" t="s">
+      <c r="AD22" s="9" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="23" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AH22" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AI22" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AQ22" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="AR22" t="s">
+        <v>59</v>
+      </c>
+      <c r="AS22" t="s">
+        <v>60</v>
+      </c>
+      <c r="AT22" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="AZ22" s="13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X23" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="AA23" t="s">
         <v>38</v>
       </c>
-      <c r="AD23" s="5" t="s">
+      <c r="AD23" s="9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="24" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AH23" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI23" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT23" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ23" s="13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X24" s="8"/>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
-      <c r="AD24" s="5" t="s">
+      <c r="AD24" s="11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="25" spans="21:30" x14ac:dyDescent="0.25">
-      <c r="AD25" s="6" t="s">
+      <c r="AI24" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>48</v>
+      </c>
+      <c r="AQ24" t="s">
+        <v>92</v>
+      </c>
+      <c r="AT24" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X25" s="8"/>
+      <c r="AD25" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="26" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AM25" t="s">
+        <v>49</v>
+      </c>
+      <c r="AQ25" s="12"/>
+      <c r="AT25" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="AZ25" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="BA25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X26" s="8"/>
       <c r="AA26" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="27" spans="21:30" x14ac:dyDescent="0.25">
+      <c r="AD26" s="10"/>
+      <c r="AH26" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI26" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="AQ26" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="AR26" t="s">
+        <v>59</v>
+      </c>
+      <c r="AS26" t="s">
+        <v>60</v>
+      </c>
+      <c r="AT26" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="AZ26" s="12"/>
+    </row>
+    <row r="27" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="X27" s="8" t="s">
+        <v>40</v>
+      </c>
       <c r="AA27" t="s">
         <v>49</v>
       </c>
-      <c r="AD27" s="5" t="s">
+      <c r="AD27" s="9" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="28" spans="21:30" x14ac:dyDescent="0.25">
-      <c r="AD28" s="5" t="s">
+      <c r="AI27" s="11" t="s">
         <v>49</v>
+      </c>
+      <c r="AQ27" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="AT27" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="AZ27" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="AD28" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AQ28" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="AT28" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="AZ28" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="AQ29" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT29" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="AZ29" s="13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="AI30" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ30" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="AZ30" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="AZ31" s="13" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="21:53" x14ac:dyDescent="0.25">
+      <c r="AQ32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="52:53" x14ac:dyDescent="0.25">
+      <c r="AZ33" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="BA33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="52:53" x14ac:dyDescent="0.25">
+      <c r="AZ34" s="12"/>
+    </row>
+    <row r="35" spans="52:53" x14ac:dyDescent="0.25">
+      <c r="AZ35" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" spans="52:53" x14ac:dyDescent="0.25">
+      <c r="AZ36" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" spans="52:53" x14ac:dyDescent="0.25">
+      <c r="AZ37" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" spans="52:53" x14ac:dyDescent="0.25">
+      <c r="AZ41" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BA41" s="6">
+        <f>SUM(BA3,BA20,BA25,BA33)</f>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>